<commit_message>
Spec gaps: consortium and subcontractor types, use of name, expenses, pricing model, modules
- Campus: consortium agreements; use-of-name clause (prior written consent)
  on research, license, collaboration, consortium and clinical trial
  playbooks; invention disclosure and royalty audit obligations
- Workforce: subcontractor addendum (flow-down of prime terms); expense
  reimbursement caps; service levels on SOWs and MSAs; Net 30 payment;
  fixed fee vs time and materials read from the pricing terms; SOW
  deliverable due dates as obligations
- Contracts: purchase order number and amount, pricing model (editable)
- Organizations choose their modules (enabledModules); /govern/me narrows
  the deployment's features to them
- Sample matrix CSV and Excel carry the use-of-name rows

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/research/review-matrix.xlsx
+++ b/samples/research/review-matrix.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="122">
   <si>
     <t>Agreement type</t>
   </si>
@@ -275,6 +275,24 @@
   </si>
   <si>
     <t>maxReportsPerYear=4; fallbackReportsPerYear=12</t>
+  </si>
+  <si>
+    <t>Use of the organization's name and marks</t>
+  </si>
+  <si>
+    <t>Neither party uses the other's name, logos or marks in advertising or publicity without prior written consent; factual statements required by law or sponsor reporting are allowed.</t>
+  </si>
+  <si>
+    <t>Use limited to a factual acknowledgement of the research funding.</t>
+  </si>
+  <si>
+    <t>may use the name of the university; may use organization's name</t>
+  </si>
+  <si>
+    <t>prior written consent</t>
+  </si>
+  <si>
+    <t>Neither party shall use the name, logos or trademarks of the other in any advertising, publicity or endorsement without the other party's prior written consent, except as required by law.</t>
   </si>
   <si>
     <t>Sponsored research</t>
@@ -375,20 +393,14 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1A41B8"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -403,15 +415,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -751,759 +757,813 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="20" style="1" customWidth="1"/>
-    <col min="2" max="2" width="34" style="1" customWidth="1"/>
-    <col min="3" max="3" width="60" style="1" customWidth="1"/>
-    <col min="4" max="4" width="50" style="1" customWidth="1"/>
-    <col min="5" max="5" width="36" style="1" customWidth="1"/>
-    <col min="6" max="6" width="26" style="1" customWidth="1"/>
-    <col min="7" max="7" width="30" style="1" customWidth="1"/>
-    <col min="8" max="8" width="70" style="1" customWidth="1"/>
-    <col min="9" max="9" width="10" style="1" customWidth="1"/>
-    <col min="10" max="10" width="30" style="1" customWidth="1"/>
+    <col min="1" max="10" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" t="s">
         <v>24</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" t="s">
         <v>25</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" t="s">
         <v>18</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" t="s">
         <v>29</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" t="s">
         <v>30</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" t="s">
         <v>31</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H4" t="s">
         <v>32</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="I4" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="J4" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" t="s">
         <v>35</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" t="s">
         <v>36</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" t="s">
         <v>37</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" t="s">
         <v>38</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="I5" t="s">
         <v>18</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>40</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" t="s">
         <v>41</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" t="s">
         <v>42</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" t="s">
         <v>43</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" t="s">
         <v>44</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" t="s">
         <v>45</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6" t="s">
         <v>18</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" t="s">
         <v>48</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" t="s">
         <v>49</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" t="s">
         <v>50</v>
       </c>
-      <c r="G7" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H7" s="1" t="s">
+      <c r="G7" t="s">
+        <v>19</v>
+      </c>
+      <c r="H7" t="s">
         <v>51</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="I7" t="s">
         <v>18</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J7" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>52</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>53</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" t="s">
         <v>54</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" t="s">
         <v>55</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" t="s">
         <v>50</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" t="s">
         <v>56</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="H8" t="s">
         <v>57</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="I8" t="s">
         <v>18</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="J8" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>59</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
         <v>60</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" t="s">
         <v>61</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" t="s">
         <v>62</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" t="s">
         <v>15</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" t="s">
         <v>63</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="H9" t="s">
         <v>64</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="I9" t="s">
         <v>65</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="J9" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="A10" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>66</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>67</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" t="s">
         <v>68</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" t="s">
         <v>69</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" t="s">
         <v>15</v>
       </c>
-      <c r="G10" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H10" s="1" t="s">
+      <c r="G10" t="s">
+        <v>19</v>
+      </c>
+      <c r="H10" t="s">
         <v>70</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="I10" t="s">
         <v>65</v>
       </c>
-      <c r="J10" s="1" t="s">
+      <c r="J10" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="A11" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>71</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>72</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="1" t="s">
+      <c r="D11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" t="s">
         <v>73</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" t="s">
         <v>15</v>
       </c>
-      <c r="G11" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H11" s="1" t="s">
+      <c r="G11" t="s">
+        <v>19</v>
+      </c>
+      <c r="H11" t="s">
         <v>74</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="I11" t="s">
         <v>65</v>
       </c>
-      <c r="J11" s="1" t="s">
+      <c r="J11" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="A12" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>75</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D12" t="s">
         <v>77</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E12" t="s">
         <v>78</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="F12" t="s">
         <v>79</v>
       </c>
-      <c r="G12" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H12" s="1" t="s">
+      <c r="G12" t="s">
+        <v>19</v>
+      </c>
+      <c r="H12" t="s">
         <v>80</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="I12" t="s">
         <v>65</v>
       </c>
-      <c r="J12" s="1" t="s">
+      <c r="J12" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="A13" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>82</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" t="s">
         <v>83</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="D13" t="s">
         <v>84</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="E13" t="s">
         <v>85</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="F13" t="s">
         <v>15</v>
       </c>
-      <c r="G13" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H13" s="1" t="s">
+      <c r="G13" t="s">
+        <v>19</v>
+      </c>
+      <c r="H13" t="s">
         <v>86</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="I13" t="s">
         <v>65</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="J13" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="A14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" t="s">
         <v>88</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="C14" t="s">
         <v>89</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="D14" t="s">
         <v>90</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="E14" t="s">
         <v>91</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="F14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G14" t="s">
         <v>92</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="H14" t="s">
         <v>93</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="I14" t="s">
+        <v>65</v>
+      </c>
+      <c r="J14" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>94</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="B15" t="s">
         <v>95</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="C15" t="s">
+        <v>96</v>
+      </c>
+      <c r="D15" t="s">
+        <v>97</v>
+      </c>
+      <c r="E15" t="s">
+        <v>98</v>
+      </c>
+      <c r="F15" t="s">
+        <v>99</v>
+      </c>
+      <c r="G15" t="s">
+        <v>100</v>
+      </c>
+      <c r="H15" t="s">
+        <v>101</v>
+      </c>
+      <c r="I15" t="s">
         <v>18</v>
       </c>
-      <c r="J14" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+      <c r="J15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" t="s">
+        <v>103</v>
+      </c>
+      <c r="D16" t="s">
+        <v>104</v>
+      </c>
+      <c r="E16" t="s">
+        <v>36</v>
+      </c>
+      <c r="F16" t="s">
+        <v>99</v>
+      </c>
+      <c r="G16" t="s">
+        <v>37</v>
+      </c>
+      <c r="H16" t="s">
+        <v>105</v>
+      </c>
+      <c r="I16" t="s">
+        <v>18</v>
+      </c>
+      <c r="J16" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>94</v>
+      </c>
+      <c r="B17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" t="s">
+        <v>41</v>
+      </c>
+      <c r="E17" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" t="s">
+        <v>43</v>
+      </c>
+      <c r="G17" t="s">
+        <v>44</v>
+      </c>
+      <c r="H17" t="s">
+        <v>106</v>
+      </c>
+      <c r="I17" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>94</v>
+      </c>
+      <c r="B18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18" t="s">
+        <v>47</v>
+      </c>
+      <c r="D18" t="s">
+        <v>48</v>
+      </c>
+      <c r="E18" t="s">
+        <v>49</v>
+      </c>
+      <c r="F18" t="s">
+        <v>50</v>
+      </c>
+      <c r="G18" t="s">
+        <v>19</v>
+      </c>
+      <c r="H18" t="s">
+        <v>51</v>
+      </c>
+      <c r="I18" t="s">
+        <v>18</v>
+      </c>
+      <c r="J18" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>94</v>
+      </c>
+      <c r="B19" t="s">
+        <v>75</v>
+      </c>
+      <c r="C19" t="s">
+        <v>76</v>
+      </c>
+      <c r="D19" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19" t="s">
+        <v>78</v>
+      </c>
+      <c r="F19" t="s">
+        <v>79</v>
+      </c>
+      <c r="G19" t="s">
+        <v>19</v>
+      </c>
+      <c r="H19" t="s">
+        <v>107</v>
+      </c>
+      <c r="I19" t="s">
+        <v>18</v>
+      </c>
+      <c r="J19" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>94</v>
+      </c>
+      <c r="B20" t="s">
+        <v>82</v>
+      </c>
+      <c r="C20" t="s">
+        <v>83</v>
+      </c>
+      <c r="D20" t="s">
+        <v>84</v>
+      </c>
+      <c r="E20" t="s">
+        <v>85</v>
+      </c>
+      <c r="F20" t="s">
+        <v>99</v>
+      </c>
+      <c r="G20" t="s">
+        <v>19</v>
+      </c>
+      <c r="H20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I20" t="s">
+        <v>18</v>
+      </c>
+      <c r="J20" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>94</v>
+      </c>
+      <c r="B21" t="s">
+        <v>52</v>
+      </c>
+      <c r="C21" t="s">
+        <v>53</v>
+      </c>
+      <c r="D21" t="s">
+        <v>54</v>
+      </c>
+      <c r="E21" t="s">
+        <v>55</v>
+      </c>
+      <c r="F21" t="s">
+        <v>50</v>
+      </c>
+      <c r="G21" t="s">
+        <v>56</v>
+      </c>
+      <c r="H21" t="s">
+        <v>108</v>
+      </c>
+      <c r="I21" t="s">
+        <v>18</v>
+      </c>
+      <c r="J21" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>94</v>
+      </c>
+      <c r="B22" t="s">
+        <v>109</v>
+      </c>
+      <c r="C22" t="s">
+        <v>110</v>
+      </c>
+      <c r="D22" t="s">
+        <v>111</v>
+      </c>
+      <c r="E22" t="s">
+        <v>19</v>
+      </c>
+      <c r="F22" t="s">
+        <v>99</v>
+      </c>
+      <c r="G22" t="s">
+        <v>112</v>
+      </c>
+      <c r="H22" t="s">
+        <v>113</v>
+      </c>
+      <c r="I22" t="s">
+        <v>18</v>
+      </c>
+      <c r="J22" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>94</v>
+      </c>
+      <c r="B23" t="s">
+        <v>115</v>
+      </c>
+      <c r="C23" t="s">
+        <v>116</v>
+      </c>
+      <c r="D23" t="s">
+        <v>19</v>
+      </c>
+      <c r="E23" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23" t="s">
+        <v>99</v>
+      </c>
+      <c r="G23" t="s">
+        <v>19</v>
+      </c>
+      <c r="H23" t="s">
+        <v>117</v>
+      </c>
+      <c r="I23" t="s">
+        <v>65</v>
+      </c>
+      <c r="J23" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>94</v>
+      </c>
+      <c r="B24" t="s">
+        <v>118</v>
+      </c>
+      <c r="C24" t="s">
+        <v>119</v>
+      </c>
+      <c r="D24" t="s">
+        <v>19</v>
+      </c>
+      <c r="E24" t="s">
+        <v>120</v>
+      </c>
+      <c r="F24" t="s">
+        <v>43</v>
+      </c>
+      <c r="G24" t="s">
+        <v>19</v>
+      </c>
+      <c r="H24" t="s">
+        <v>121</v>
+      </c>
+      <c r="I24" t="s">
+        <v>65</v>
+      </c>
+      <c r="J24" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>94</v>
+      </c>
+      <c r="B25" t="s">
         <v>88</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="F15" s="1" t="s">
+      <c r="C25" t="s">
+        <v>89</v>
+      </c>
+      <c r="D25" t="s">
+        <v>90</v>
+      </c>
+      <c r="E25" t="s">
+        <v>91</v>
+      </c>
+      <c r="F25" t="s">
+        <v>50</v>
+      </c>
+      <c r="G25" t="s">
+        <v>92</v>
+      </c>
+      <c r="H25" t="s">
         <v>93</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="I20" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="I22" s="1" t="s">
+      <c r="I25" t="s">
         <v>65</v>
       </c>
-      <c r="J22" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="J23" s="1" t="s">
+      <c r="J25" t="s">
         <v>19</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>